<commit_message>
Update review summary workbook with all reviews and 3조 reference data
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014B4DRCucP2d4gQGFG2Gfdc
</commit_message>
<xml_diff>
--- a/클렌징폼_리뷰_조사요약.xlsx
+++ b/클렌징폼_리뷰_조사요약.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="비플레인" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="라운드랩" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="마녀공장" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="리뷰별 분류표" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="참고_3조 가상구매데이터" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="리뷰별 분류표" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +48,11 @@
     <font>
       <color rgb="FF777777"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF6D2E46"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="5">
@@ -98,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,6 +121,8 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -495,7 +503,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>조사 요약 시트 — 우리 조가 직접 쓰는 '조사 요약' (전체 38개)</t>
+          <t>조사 요약 시트 — 우리 조가 직접 쓰는 '조사 요약' (전체 43개)</t>
         </is>
       </c>
     </row>
@@ -544,8 +552,8 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>리뷰 38개 중 24개 언급 (63%) · 비플레인 8 라운드랩 6 마녀공장 10
-No 1, 2, 3, 5, 13, 15, 18, 19, 20, 21, 23, 26, 27, 28, 30, 31, 32, 33, 34, 35, 38, 39, 40, 41</t>
+          <t>리뷰 43개 중 29개 언급 (67%) · 비플레인 8 라운드랩 11 마녀공장 10
+No 1, 2, 3, 5, 13, 15, 18, 19, 20, 21, 23, 26, 27, 28, 42, 43, 44, 45, 46, 30, 31, 32, 33, 34, 35, 38, 39, 40, 41</t>
         </is>
       </c>
     </row>
@@ -561,8 +569,8 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>리뷰 38개 중 24개 언급 (63%) · 비플레인 13 라운드랩 4 마녀공장 7
-No 2, 3, 4, 5, 6, 7, 9, 10, 12, 13, 17, 18, 19, 20, 21, 24, 26, 32, 33, 34, 35, 36, 40, 41</t>
+          <t>리뷰 43개 중 27개 언급 (63%) · 비플레인 13 라운드랩 7 마녀공장 7
+No 2, 3, 4, 5, 6, 7, 9, 10, 12, 13, 17, 18, 19, 20, 21, 24, 26, 43, 45, 46, 32, 33, 34, 35, 36, 40, 41</t>
         </is>
       </c>
     </row>
@@ -578,8 +586,8 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>리뷰 38개 중 14개 언급 (37%) · 비플레인 4 라운드랩 5 마녀공장 5
-No 3, 6, 7, 14, 20, 21, 25, 26, 28, 32, 34, 37, 38, 41</t>
+          <t>리뷰 43개 중 15개 언급 (35%) · 비플레인 4 라운드랩 6 마녀공장 5
+No 3, 6, 7, 14, 20, 21, 25, 26, 28, 45, 32, 34, 37, 38, 41</t>
         </is>
       </c>
     </row>
@@ -599,8 +607,8 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>리뷰 38개 중 6개 언급 (16%) · 비플레인 4 라운드랩 0 마녀공장 2
-No 2, 5, 13, 18, 36, 41</t>
+          <t>리뷰 43개 중 7개 언급 (16%) · 비플레인 4 라운드랩 1 마녀공장 2
+No 2, 5, 13, 18, 36, 41, 45</t>
         </is>
       </c>
     </row>
@@ -616,8 +624,8 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>리뷰 38개 중 5개 언급 (13%) · 비플레인 2 라운드랩 2 마녀공장 1
-No 7, 15, 22, 24, 36</t>
+          <t>리뷰 43개 중 6개 언급 (14%) · 비플레인 2 라운드랩 3 마녀공장 1
+No 7, 15, 22, 24, 36, 45</t>
         </is>
       </c>
     </row>
@@ -628,13 +636,13 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>후기·커뮤니티 글 참고</t>
+          <t>성분 확인 (화해 앱 등)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>리뷰 38개 중 4개 언급 (11%) · 비플레인 3 라운드랩 1 마녀공장 0
-No 6, 13, 17, 26</t>
+          <t>리뷰 43개 중 5개 언급 (12%) · 비플레인 3 라운드랩 2 마녀공장 0
+No 2, 5, 9, 45, 46</t>
         </is>
       </c>
     </row>
@@ -654,8 +662,8 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>리뷰 38개 중 25개 언급 (66%) · 비플레인 11 라운드랩 5 마녀공장 9
-No 2, 4, 5, 6, 7, 9, 10, 12, 13, 17, 19, 21, 22, 24, 26, 27, 30, 32, 33, 34, 35, 36, 39, 40, 41</t>
+          <t>리뷰 43개 중 30개 언급 (70%) · 비플레인 11 라운드랩 10 마녀공장 9
+No 2, 4, 5, 6, 7, 9, 10, 12, 13, 17, 19, 21, 22, 24, 26, 27, 42, 43, 44, 45, 46, 30, 32, 33, 34, 35, 36, 39, 40, 41</t>
         </is>
       </c>
     </row>
@@ -671,8 +679,8 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>리뷰 38개 중 24개 언급 (63%) · 비플레인 11 라운드랩 5 마녀공장 8
-No 1, 2, 3, 5, 6, 7, 10, 14, 15, 18, 19, 20, 21, 23, 25, 28, 29, 30, 31, 32, 34, 37, 38, 41</t>
+          <t>리뷰 43개 중 27개 언급 (63%) · 비플레인 11 라운드랩 8 마녀공장 8
+No 1, 2, 3, 5, 6, 7, 10, 14, 15, 18, 19, 20, 21, 23, 25, 28, 42, 45, 46, 29, 30, 31, 32, 34, 37, 38, 41</t>
         </is>
       </c>
     </row>
@@ -688,8 +696,8 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>리뷰 38개 중 19개 언급 (50%) · 비플레인 8 라운드랩 3 마녀공장 8
-No 2, 3, 7, 10, 12, 13, 14, 15, 23, 25, 26, 31, 32, 33, 34, 37, 38, 40, 41</t>
+          <t>리뷰 43개 중 20개 언급 (47%) · 비플레인 8 라운드랩 4 마녀공장 8
+No 2, 3, 7, 10, 12, 13, 14, 15, 23, 25, 26, 45, 31, 32, 33, 34, 37, 38, 40, 41</t>
         </is>
       </c>
     </row>
@@ -958,7 +966,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>리뷰 9개 기준</t>
+          <t>리뷰 14개 기준</t>
         </is>
       </c>
     </row>
@@ -1000,8 +1008,8 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>리뷰 9개 중 6개 언급 (67%)
-No 20, 21, 23, 26, 27, 28</t>
+          <t>리뷰 14개 중 11개 언급 (79%)
+No 20, 21, 23, 26, 27, 28, 42, 43, 44, 45, 46</t>
         </is>
       </c>
     </row>
@@ -1012,13 +1020,13 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>잔여감·미끄덩함</t>
+          <t>피부 자극·트러블 반응</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>리뷰 9개 중 5개 언급 (56%)
-No 20, 21, 25, 26, 28</t>
+          <t>리뷰 14개 중 7개 언급 (50%)
+No 20, 21, 24, 26, 43, 45, 46</t>
         </is>
       </c>
     </row>
@@ -1029,13 +1037,13 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>피부 자극·트러블 반응</t>
+          <t>잔여감·미끄덩함</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>리뷰 9개 중 4개 언급 (44%)
-No 20, 21, 24, 26</t>
+          <t>리뷰 14개 중 6개 언급 (43%)
+No 20, 21, 25, 26, 28, 45</t>
         </is>
       </c>
     </row>
@@ -1055,8 +1063,8 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>리뷰 9개 중 2개 언급 (22%)
-No 22, 24</t>
+          <t>리뷰 14개 중 3개 언급 (21%)
+No 22, 24, 45</t>
         </is>
       </c>
     </row>
@@ -1067,13 +1075,13 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>후기·커뮤니티 글 참고</t>
+          <t>성분 확인 (화해 앱 등)</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>리뷰 9개 중 1개 언급 (11%)
-No 26</t>
+          <t>리뷰 14개 중 2개 언급 (14%)
+No 45, 46</t>
         </is>
       </c>
     </row>
@@ -1084,12 +1092,13 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>해당 없음 (언급 리뷰 없음)</t>
+          <t>문제 인식 후 순한·약산성 제품 탐색</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>리뷰 14개 중 1개 언급 (7%)
+No 45</t>
         </is>
       </c>
     </row>
@@ -1109,8 +1118,8 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>리뷰 9개 중 5개 언급 (56%)
-No 21, 22, 24, 26, 27</t>
+          <t>리뷰 14개 중 10개 언급 (71%)
+No 21, 22, 24, 26, 27, 42, 43, 44, 45, 46</t>
         </is>
       </c>
     </row>
@@ -1126,8 +1135,8 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>리뷰 9개 중 5개 언급 (56%)
-No 20, 21, 23, 25, 28</t>
+          <t>리뷰 14개 중 8개 언급 (57%)
+No 20, 21, 23, 25, 28, 42, 45, 46</t>
         </is>
       </c>
     </row>
@@ -1138,13 +1147,13 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>풍성·부드러운 거품</t>
+          <t>가격·용량·구성</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>리뷰 9개 중 3개 언급 (33%)
-No 23, 25, 26</t>
+          <t>리뷰 14개 중 6개 언급 (43%)
+No 24, 42, 43, 44, 45, 46</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1402,464 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q39"/>
+  <dimension ref="A1:C39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>참고 — 3조_클렌징 가상 구매 고객 50명 (가상 데이터, 리뷰와 합산하지 않음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>실제 리뷰가 아닌 수업용 가상 멤버십 데이터. 리뷰에서 근거가 약한 정보 탐색·채널 항목의 참고용.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>첫 구매 유입 경로(정보 탐색)</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>고객 수</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>비중(%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>숏폼·SNS</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>유튜브 리뷰</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>지인 추천</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>성분 검색·성분 앱</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>매장 진열·직원 추천</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>커뮤니티·리뷰</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>피부과·약사 권유</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>주 구매 채널</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>고객 수</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>비중(%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>올리브영 앱</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>14</v>
+      </c>
+      <c r="C14" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>올리브영 매장</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>13</v>
+      </c>
+      <c r="C15" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>온라인 종합몰</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>12</v>
+      </c>
+      <c r="C16" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>다이소</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>약국·병의원</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>브랜드 자사몰</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>대표 피부 고민</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>고객 수</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>비중(%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>모공·블랙헤드</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>13</v>
+      </c>
+      <c r="C22" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>세안 귀찮음</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>11</v>
+      </c>
+      <c r="C23" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>메이크업 잔여감</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>10</v>
+      </c>
+      <c r="C24" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>세안 후 당김</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>6</v>
+      </c>
+      <c r="C25" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>트러블</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>6</v>
+      </c>
+      <c r="C26" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>자극·따가움</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>주 구매 제품 유형</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>고객 수</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>비중(%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>클렌징 오일</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>12</v>
+      </c>
+      <c r="C30" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>약산성 젤 클렌저</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>7</v>
+      </c>
+      <c r="C31" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>클렌징 워터</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C32" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>클렌징 티슈</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>6</v>
+      </c>
+      <c r="C33" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>올인원 폼</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>6</v>
+      </c>
+      <c r="C34" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>클렌징 밤</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>6</v>
+      </c>
+      <c r="C35" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>클렌징 밀크</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>클렌징 폼</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>동일 제품 재구매 Y 46/50 · 평균 연령 27.2세 · 연 구매 7.2회 · 평균 단가 16,056원 · 세일 구매 비중 평균 49.5% · 대용량·리필 25/50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1416,87 +1882,87 @@
   </cols>
   <sheetData>
     <row r="1" ht="60" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>제품</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="10" t="inlineStr">
         <is>
           <t>건조함·당김</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>피부 자극·트러블 반응</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>잔여감·미끄덩함</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="10" t="inlineStr">
         <is>
           <t>거품 부족·약함</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="G1" s="10" t="inlineStr">
         <is>
           <t>세정력 부족</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="H1" s="10" t="inlineStr">
         <is>
           <t>냄새·향 불만</t>
         </is>
       </c>
-      <c r="I1" s="8" t="inlineStr">
+      <c r="I1" s="10" t="inlineStr">
         <is>
           <t>문제 인식 후 순한·약산성 제품 탐색</t>
         </is>
       </c>
-      <c r="J1" s="8" t="inlineStr">
+      <c r="J1" s="10" t="inlineStr">
         <is>
           <t>추천·조언 (지인·직원·유튜버)</t>
         </is>
       </c>
-      <c r="K1" s="8" t="inlineStr">
+      <c r="K1" s="10" t="inlineStr">
         <is>
           <t>후기·커뮤니티 글 참고</t>
         </is>
       </c>
-      <c r="L1" s="8" t="inlineStr">
+      <c r="L1" s="10" t="inlineStr">
         <is>
           <t>성분 확인 (화해 앱 등)</t>
         </is>
       </c>
-      <c r="M1" s="8" t="inlineStr">
+      <c r="M1" s="10" t="inlineStr">
         <is>
           <t>같은 브랜드 타 제품 사용 후 교차 구매</t>
         </is>
       </c>
-      <c r="N1" s="8" t="inlineStr">
+      <c r="N1" s="10" t="inlineStr">
         <is>
           <t>저자극·순한 사용감 (자극·당김 적음)</t>
         </is>
       </c>
-      <c r="O1" s="8" t="inlineStr">
+      <c r="O1" s="10" t="inlineStr">
         <is>
           <t>세정력·마무리감 (뽀득·개운·잔여감)</t>
         </is>
       </c>
-      <c r="P1" s="8" t="inlineStr">
+      <c r="P1" s="10" t="inlineStr">
         <is>
           <t>풍성·부드러운 거품</t>
         </is>
       </c>
-      <c r="Q1" s="8" t="inlineStr">
+      <c r="Q1" s="10" t="inlineStr">
         <is>
           <t>가격·용량·구성</t>
         </is>
@@ -2609,14 +3075,18 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>마녀공장</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
+          <t>라운드랩</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -2627,22 +3097,30 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
       <c r="O27" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
       <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>마녀공장</t>
+          <t>라운드랩</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2650,7 +3128,11 @@
           <t>●</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
@@ -2665,21 +3147,21 @@
           <t>●</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>마녀공장</t>
+          <t>라운드랩</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2697,17 +3179,13 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr">
         <is>
           <t>●</t>
@@ -2716,11 +3194,11 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>마녀공장</t>
+          <t>라운드랩</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2741,10 +3219,22 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
@@ -2761,15 +3251,19 @@
           <t>●</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>마녀공장</t>
+          <t>라운드랩</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2783,51 +3277,51 @@
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr"/>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
           <t>마녀공장</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
@@ -2836,30 +3330,18 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2871,11 +3353,7 @@
           <t>●</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
@@ -2890,62 +3368,74 @@
           <t>●</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
           <t>마녀공장</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
           <t>마녀공장</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>●</t>
@@ -2959,7 +3449,11 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
       <c r="O35" t="inlineStr">
         <is>
           <t>●</t>
@@ -2970,15 +3464,11 @@
           <t>●</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="Q35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2990,12 +3480,12 @@
           <t>●</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
@@ -3004,26 +3494,22 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="Q36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3035,8 +3521,16 @@
           <t>●</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
@@ -3050,8 +3544,16 @@
           <t>●</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
       <c r="Q37" t="inlineStr">
         <is>
           <t>●</t>
@@ -3060,7 +3562,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3092,37 +3594,25 @@
         </is>
       </c>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
           <t>마녀공장</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
+      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
@@ -3131,7 +3621,11 @@
           <t>●</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
@@ -3140,17 +3634,226 @@
           <t>●</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>마녀공장</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>마녀공장</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>마녀공장</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>마녀공장</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>마녀공장</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
         <is>
           <t>●</t>
         </is>

</xml_diff>